<commit_message>
Mapping updates and additions
Existing mappings updated after several improvements and additions. Added mappings for BRO objects BHR, GUF and GPD
</commit_message>
<xml_diff>
--- a/BROMappings/Mapping BRO GLD Events.xlsx
+++ b/BROMappings/Mapping BRO GLD Events.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://3hydro-my.sharepoint.com/personal/jos_von_asmuth_3hydro_nl/Documents/MATLAB/Menyanthes/Meny_OS/trunk/Datamodels/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://3hydro-my.sharepoint.com/personal/jos_von_asmuth_3hydro_nl/Documents/MATLAB/Menyanthes/Meny_OS/trunk/BronDatamodel/BROMappings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="68" documentId="13_ncr:1_{095261ED-ABE2-49B7-9BF7-3FCA8EA64B04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4C362502-4182-4FAB-B2CA-FA91D5DEBAB6}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{6C14A7D8-3620-4B60-882E-67C4BBD26BE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4AB0629-70FA-4C08-8C28-1C0BC5696D4F}"/>
   <bookViews>
-    <workbookView xWindow="-3810" yWindow="3930" windowWidth="23250" windowHeight="11655" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="53">
   <si>
     <t>BROBrondocument</t>
   </si>
@@ -54,12 +54,6 @@
     <t>BROGebeurtenisData</t>
   </si>
   <si>
-    <t>BROGebeurtenisWerkafspraak</t>
-  </si>
-  <si>
-    <t>BROGebeurtenisNieuw</t>
-  </si>
-  <si>
     <t>Correctie (attribuut)</t>
   </si>
   <si>
@@ -166,22 +160,38 @@
   </si>
   <si>
     <t>De BRO maakt geen onderscheid tussen correcties van attribuutwaarden en metingen</t>
+  </si>
+  <si>
+    <t>[Categorical]</t>
+  </si>
+  <si>
+    <t>[String]</t>
+  </si>
+  <si>
+    <t>BronOmschrijving</t>
+  </si>
+  <si>
+    <t>Beoordelen</t>
+  </si>
+  <si>
+    <t>Metingen beoordeeld</t>
+  </si>
+  <si>
+    <t>GLD_Status</t>
+  </si>
+  <si>
+    <t>GLD-Beoordeling</t>
+  </si>
+  <si>
+    <t>GLD_Status is geen echt brondocument, maar een optie. Indien een observatie voorlopig geregistreerd was, dan betreft dit een vervangverzoek. Zo niet, dan betreft het een aanvulling. Het betreft alle observaties tot dan toe in eens</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -201,16 +211,42 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF005E6A"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF85C9EB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="18">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -229,103 +265,6 @@
     </border>
     <border>
       <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="medium">
         <color indexed="64"/>
       </right>
@@ -365,19 +304,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -422,6 +348,76 @@
         <color indexed="64"/>
       </right>
       <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom style="thin">
@@ -433,36 +429,49 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -478,10 +487,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -747,247 +752,263 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="30.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="31.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.5703125" customWidth="1"/>
-    <col min="7" max="7" width="102.5703125" customWidth="1"/>
+    <col min="4" max="4" width="23.5703125" customWidth="1"/>
+    <col min="5" max="5" width="62.85546875" customWidth="1"/>
+    <col min="6" max="6" width="107.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="B1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="F1" s="14" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="D2" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="E2" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" s="2"/>
+      <c r="F3" s="6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" t="s">
+        <v>39</v>
+      </c>
+      <c r="F4" s="4"/>
+    </row>
+    <row r="5" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" t="s">
+        <v>40</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" s="2"/>
+      <c r="F6" s="6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" s="2"/>
+      <c r="F8" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A9" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="B9" s="22" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="D9" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="E9" s="21"/>
+      <c r="F9" s="23" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="F10" s="4"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" t="s">
+        <v>43</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" t="s">
+        <v>18</v>
+      </c>
+      <c r="F12" s="4"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D13" t="s">
+        <v>19</v>
+      </c>
+      <c r="F13" s="4"/>
+    </row>
+    <row r="14" spans="1:6" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="F1" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="G1" s="9" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="G2" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="21" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17" t="s">
-        <v>41</v>
-      </c>
-      <c r="G3" s="11"/>
-    </row>
-    <row r="4" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="21" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="17" t="s">
+      <c r="E14" s="7"/>
+      <c r="F14" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="G4" s="12" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="22" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="G5" s="13" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="21" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="C6" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17" t="s">
-        <v>38</v>
-      </c>
-      <c r="G6" s="11" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G7" s="13" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="21" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="C8" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="G8" s="11"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="21" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="C9" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="G9" s="11" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="21" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="17" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="G10" s="11"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="21" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="G11" s="11"/>
-    </row>
-    <row r="12" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" s="20" t="s">
-        <v>4</v>
-      </c>
-      <c r="C12" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="G12" s="15" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B13" s="1"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B14" s="1"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B15" s="1"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B16" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>